<commit_message>
refactor(config): remove unused fallback models from agent configurations
Clean up agent configuration by removing deprecated and unused fallback model
entries (qwen3.7-plus, kimi-k2.7-code, kimi-k2.6, nemotron-3-ultra-free,
north-mini-code-free) from multiple agent profiles to streamline the model
fallback chain and reduce configuration complexity.
</commit_message>
<xml_diff>
--- a/OpenCode/OpencodeModels.xlsx
+++ b/OpenCode/OpencodeModels.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Configs_Agents\OpenCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A16487-2AB6-467A-B4CA-E32782B0243B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADE6403-4530-4FAF-92D8-0339E94B72EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Artificial Analysis" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="33">
   <si>
     <t>requests per 5 hour</t>
   </si>
@@ -50,9 +51,6 @@
     <t>GLM-5.1</t>
   </si>
   <si>
-    <t>GLM-5</t>
-  </si>
-  <si>
     <t>Kimi K2.6</t>
   </si>
   <si>
@@ -116,7 +114,28 @@
     <t>norm</t>
   </si>
   <si>
-    <t>MiniMax M3 (3x)</t>
+    <t>GLM-5.2</t>
+  </si>
+  <si>
+    <t>GLM-5.2 (max)</t>
+  </si>
+  <si>
+    <t>MiniMax-M3</t>
+  </si>
+  <si>
+    <t>DeepSeek V4 Pro (max)</t>
+  </si>
+  <si>
+    <t>DeepSeek V4 Flash (max)</t>
+  </si>
+  <si>
+    <t>MiniMax-M2.7</t>
+  </si>
+  <si>
+    <t>Intelligence</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -163,18 +182,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="14">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
@@ -186,9 +228,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="166" formatCode="0.0"/>
@@ -219,35 +258,51 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CC3859BB-9B9A-4EC2-A38E-BACA98F6B13E}" name="Table1" displayName="Table1" ref="A1:K15" totalsRowShown="0">
-  <autoFilter ref="A1:K15" xr:uid="{CC3859BB-9B9A-4EC2-A38E-BACA98F6B13E}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K15">
-    <sortCondition descending="1" ref="K1:K15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CC3859BB-9B9A-4EC2-A38E-BACA98F6B13E}" name="Table1" displayName="Table1" ref="A1:L14" totalsRowShown="0">
+  <autoFilter ref="A1:L14" xr:uid="{CC3859BB-9B9A-4EC2-A38E-BACA98F6B13E}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L14">
+    <sortCondition descending="1" ref="L1:L14"/>
   </sortState>
-  <tableColumns count="11">
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{4558084D-BFD3-4096-990D-BABDB4A3F9A5}" name="Model"/>
-    <tableColumn id="2" xr3:uid="{77DF4AD7-27A3-4A22-84ED-536798D59DFB}" name="requests per 5 hour" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{968D85ED-4421-4AB0-AE6D-E50ECE878D7F}" name="requests per week" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{389CEFA6-A786-416D-9098-1BF29A227B30}" name="requests per month" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{98FE1845-9B6F-44C3-A0B3-7C65A82D1700}" name="norm kota 5" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{77DF4AD7-27A3-4A22-84ED-536798D59DFB}" name="requests per 5 hour" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{968D85ED-4421-4AB0-AE6D-E50ECE878D7F}" name="requests per week" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{389CEFA6-A786-416D-9098-1BF29A227B30}" name="requests per month" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{98FE1845-9B6F-44C3-A0B3-7C65A82D1700}" name="norm kota 5" dataDxfId="10">
       <calculatedColumnFormula>(Table1[[#This Row],[requests per month]]-MIN(Table1[requests per month]))/(MAX(Table1[requests per month])-MIN(Table1[requests per month]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{5D7E2A26-E549-4CFD-B043-F0481B5110F6}" name="EK böl kota 6" dataDxfId="5">
+    <tableColumn id="12" xr3:uid="{5D7E2A26-E549-4CFD-B043-F0481B5110F6}" name="EK böl kota 6" dataDxfId="9">
       <calculatedColumnFormula>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{D33AC59D-2F81-400A-BD0D-DB990B819EAB}" name="Coding" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{9BC67038-D32E-487A-B892-E1CBD2D5A5C1}" name="norm kod" dataDxfId="3">
+    <tableColumn id="6" xr3:uid="{EB1EE3D7-51B5-45D4-94BD-7E18987D18E7}" name="Intelligence" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{D33AC59D-2F81-400A-BD0D-DB990B819EAB}" name="Coding" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{9BC67038-D32E-487A-B892-E1CBD2D5A5C1}" name="norm kod" dataDxfId="8">
       <calculatedColumnFormula>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{1DBCEBD9-B051-4EC1-871D-57D21FFF0BCC}" name="EK Böl Kod" dataDxfId="2">
+    <tableColumn id="13" xr3:uid="{1DBCEBD9-B051-4EC1-871D-57D21FFF0BCC}" name="EK Böl Kod" dataDxfId="7">
       <calculatedColumnFormula>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{EDE10E07-3FEB-4504-8C05-B05E66499132}" name="norm" dataDxfId="1">
-      <calculatedColumnFormula>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</calculatedColumnFormula>
+    <tableColumn id="10" xr3:uid="{EDE10E07-3FEB-4504-8C05-B05E66499132}" name="norm" dataDxfId="6">
+      <calculatedColumnFormula>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{3B61D66B-5DEA-4B74-AF9F-DE1BA05DA990}" name="Column1" dataDxfId="0">
+    <tableColumn id="14" xr3:uid="{3B61D66B-5DEA-4B74-AF9F-DE1BA05DA990}" name="Column1" dataDxfId="5">
       <calculatedColumnFormula>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</calculatedColumnFormula>
     </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B1A2C6D8-E425-48A2-9791-4CC58FDD9323}" name="Table3" displayName="Table3" ref="A1:C14" totalsRowShown="0">
+  <autoFilter ref="A1:C14" xr:uid="{B1A2C6D8-E425-48A2-9791-4CC58FDD9323}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C14">
+    <sortCondition ref="A1:A14"/>
+  </sortState>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{F70AD1CB-BF1B-456C-89F9-F7F05A62C0B2}" name="Model" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{AB274D46-C44C-4532-B610-E18FDE2EDCA8}" name="Intelligence" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{68060333-0096-47A0-B7E1-CC2B0C9BC864}" name="Coding" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -516,22 +571,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.44140625" customWidth="1"/>
     <col min="5" max="5" width="9.109375" customWidth="1"/>
     <col min="6" max="6" width="10.44140625" customWidth="1"/>
-    <col min="7" max="8" width="10.77734375" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" customWidth="1"/>
+    <col min="9" max="10" width="10.77734375" customWidth="1"/>
+    <col min="11" max="11" width="10.88671875" customWidth="1"/>
+    <col min="12" max="12" width="12.109375" customWidth="1"/>
+    <col min="13" max="13" width="13.6640625" customWidth="1"/>
+    <col min="15" max="15" width="12.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -543,30 +599,33 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
         <v>22</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1" t="s">
         <v>23</v>
       </c>
-      <c r="G1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H1" t="s">
-        <v>21</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1">
         <v>30100</v>
@@ -585,358 +644,384 @@
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
         <v>34.97674418604651</v>
       </c>
-      <c r="G2" s="2">
-        <v>42.1</v>
-      </c>
-      <c r="H2" s="3">
+      <c r="G2" s="6">
+        <v>40</v>
+      </c>
+      <c r="H2" s="6">
+        <v>60.7</v>
+      </c>
+      <c r="I2" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0.29824561403508765</v>
-      </c>
-      <c r="I2" s="2">
+        <v>0.50000000000000022</v>
+      </c>
+      <c r="J2" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.0878552971576227</v>
-      </c>
-      <c r="J2" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.62393593668930203</v>
+        <v>1.1539923954372624</v>
       </c>
       <c r="K2" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>0.72481312967175837</v>
+      </c>
+      <c r="L2" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>1854705.2757296057</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+        <v>3593392.6540494892</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
       <c r="B3" s="1">
-        <v>3450</v>
+        <v>31650</v>
       </c>
       <c r="C3" s="1">
-        <v>8550</v>
+        <v>79050</v>
       </c>
       <c r="D3" s="1">
-        <v>17150</v>
+        <v>158150</v>
       </c>
       <c r="E3" s="4">
         <f>(Table1[[#This Row],[requests per month]]-MIN(Table1[requests per month]))/(MAX(Table1[requests per month])-MIN(Table1[requests per month]))</f>
-        <v>8.3522911927201821E-2</v>
+        <v>1</v>
       </c>
       <c r="F3" s="5">
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
-        <v>3.9883720930232558</v>
-      </c>
-      <c r="G3" s="2">
-        <v>47.5</v>
-      </c>
-      <c r="H3" s="3">
+        <v>36.779069767441861</v>
+      </c>
+      <c r="G3" s="6">
+        <v>40</v>
+      </c>
+      <c r="H3" s="6">
+        <v>56.2</v>
+      </c>
+      <c r="I3" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0.77192982456140335</v>
-      </c>
-      <c r="I3" s="2">
+        <v>0.22222222222222238</v>
+      </c>
+      <c r="J3" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.2273901808785528</v>
-      </c>
-      <c r="J3" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.4277263682443026</v>
+        <v>1.0684410646387832</v>
       </c>
       <c r="K3" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>0.61111111111111116</v>
+      </c>
+      <c r="L3" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>853657.17666450515</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+        <v>1606132.3397738335</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="B4" s="1">
+        <v>880</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2150</v>
+      </c>
+      <c r="D4" s="1">
         <v>4300</v>
-      </c>
-      <c r="C4" s="1">
-        <v>10800</v>
-      </c>
-      <c r="D4" s="1">
-        <v>21600</v>
       </c>
       <c r="E4" s="4">
         <f>(Table1[[#This Row],[requests per month]]-MIN(Table1[requests per month]))/(MAX(Table1[requests per month])-MIN(Table1[requests per month]))</f>
-        <v>0.11244718882027949</v>
+        <v>0</v>
       </c>
       <c r="F4" s="5">
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
-        <v>5.0232558139534884</v>
-      </c>
-      <c r="G4" s="2">
-        <v>46.5</v>
-      </c>
-      <c r="H4" s="3">
+        <v>1</v>
+      </c>
+      <c r="G4" s="6">
+        <v>51</v>
+      </c>
+      <c r="H4" s="6">
+        <v>68.8</v>
+      </c>
+      <c r="I4" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0.68421052631578927</v>
-      </c>
-      <c r="I4" s="2">
+        <v>1</v>
+      </c>
+      <c r="J4" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.2015503875968991</v>
-      </c>
-      <c r="J4" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.39832885756803438</v>
+        <v>1.3079847908745246</v>
       </c>
       <c r="K4" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>0.5</v>
+      </c>
+      <c r="L4" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>830333.05299905303</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+        <v>479187.82031011395</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="B5" s="1">
-        <f>3*3200</f>
-        <v>9600</v>
+        <v>3250</v>
       </c>
       <c r="C5" s="1">
-        <f>3*8000</f>
-        <v>24000</v>
+        <v>8150</v>
       </c>
       <c r="D5" s="1">
-        <f>3*16000</f>
-        <v>48000</v>
+        <v>16300</v>
       </c>
       <c r="E5" s="4">
         <f>(Table1[[#This Row],[requests per month]]-MIN(Table1[requests per month]))/(MAX(Table1[requests per month])-MIN(Table1[requests per month]))</f>
-        <v>0.28404289892752682</v>
+        <v>7.7998050048748782E-2</v>
       </c>
       <c r="F5" s="5">
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
-        <v>11.162790697674419</v>
-      </c>
-      <c r="G5" s="2">
-        <v>43.4</v>
-      </c>
-      <c r="H5" s="3">
+        <v>3.7906976744186047</v>
+      </c>
+      <c r="G5" s="6">
+        <v>42</v>
+      </c>
+      <c r="H5" s="6">
+        <v>60.2</v>
+      </c>
+      <c r="I5" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0.41228070175438564</v>
-      </c>
-      <c r="I5" s="2">
+        <v>0.469135802469136</v>
+      </c>
+      <c r="J5" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.1214470284237725</v>
-      </c>
-      <c r="J5" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.34816180034095623</v>
+        <v>1.1444866920152093</v>
       </c>
       <c r="K5" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>0.27356692625894241</v>
+      </c>
+      <c r="L5" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>828238.36506090988</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>354129.1674144339</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1">
-        <v>1350</v>
+        <v>3450</v>
       </c>
       <c r="C6" s="1">
-        <v>4630</v>
+        <v>8550</v>
       </c>
       <c r="D6" s="1">
-        <v>9250</v>
+        <v>17150</v>
       </c>
       <c r="E6" s="4">
         <f>(Table1[[#This Row],[requests per month]]-MIN(Table1[requests per month]))/(MAX(Table1[requests per month])-MIN(Table1[requests per month]))</f>
-        <v>3.2174195645108872E-2</v>
+        <v>8.3522911927201821E-2</v>
       </c>
       <c r="F6" s="5">
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
-        <v>2.1511627906976742</v>
-      </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="3">
+        <v>3.9883720930232558</v>
+      </c>
+      <c r="G6" s="6">
+        <v>44</v>
+      </c>
+      <c r="H6" s="6">
+        <v>59.4</v>
+      </c>
+      <c r="I6" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>-3.3947368421052637</v>
-      </c>
-      <c r="I6" s="2">
+        <v>0.41975308641975301</v>
+      </c>
+      <c r="J6" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>0</v>
-      </c>
-      <c r="J6" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>-1.6812813232300774</v>
+        <v>1.1292775665399239</v>
       </c>
       <c r="K6" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>0.2516379991734774</v>
+      </c>
+      <c r="L6" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>2.1511627906976742</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+        <v>320026.41438157106</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B7" s="1">
-        <v>31650</v>
+        <v>950</v>
       </c>
       <c r="C7" s="1">
-        <v>79050</v>
+        <v>2390</v>
       </c>
       <c r="D7" s="1">
-        <v>158150</v>
+        <v>4770</v>
       </c>
       <c r="E7" s="4">
         <f>(Table1[[#This Row],[requests per month]]-MIN(Table1[requests per month]))/(MAX(Table1[requests per month])-MIN(Table1[requests per month]))</f>
-        <v>1</v>
+        <v>3.0549236269093272E-3</v>
       </c>
       <c r="F7" s="5">
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
-        <v>36.779069767441861</v>
-      </c>
-      <c r="G7" s="2">
-        <v>38.700000000000003</v>
-      </c>
-      <c r="H7" s="3">
+        <v>1.1093023255813954</v>
+      </c>
+      <c r="G7" s="6">
+        <v>46</v>
+      </c>
+      <c r="H7" s="6">
+        <v>66</v>
+      </c>
+      <c r="I7" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0</v>
-      </c>
-      <c r="I7" s="2">
+        <v>0.82716049382716061</v>
+      </c>
+      <c r="J7" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1</v>
-      </c>
-      <c r="J7" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.5</v>
+        <v>1.2547528517110267</v>
       </c>
       <c r="K7" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>0.41510770872703495</v>
+      </c>
+      <c r="L7" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>810112.922197368</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+        <v>312156.45496074983</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="1">
-        <v>3250</v>
+        <v>3200</v>
       </c>
       <c r="C8" s="1">
-        <v>8150</v>
+        <v>8000</v>
       </c>
       <c r="D8" s="1">
-        <v>16300</v>
+        <v>16000</v>
       </c>
       <c r="E8" s="4">
         <f>(Table1[[#This Row],[requests per month]]-MIN(Table1[requests per month]))/(MAX(Table1[requests per month])-MIN(Table1[requests per month]))</f>
-        <v>7.7998050048748782E-2</v>
+        <v>7.6048098797530064E-2</v>
       </c>
       <c r="F8" s="5">
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
-        <v>3.7906976744186047</v>
-      </c>
-      <c r="G8" s="2">
-        <v>45.5</v>
-      </c>
-      <c r="H8" s="3">
+        <v>3.7209302325581395</v>
+      </c>
+      <c r="G8" s="6">
+        <v>44</v>
+      </c>
+      <c r="H8" s="6">
+        <v>58.6</v>
+      </c>
+      <c r="I8" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0.59649122807017529</v>
-      </c>
-      <c r="I8" s="2">
+        <v>0.37037037037037046</v>
+      </c>
+      <c r="J8" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.1757105943152455</v>
-      </c>
-      <c r="J8" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.33724463905946206</v>
+        <v>1.1140684410646389</v>
       </c>
       <c r="K8" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>0.22320923458395026</v>
+      </c>
+      <c r="L8" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>483910.87600904744</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+        <v>256442.08027163282</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9">
-        <v>950</v>
+        <v>5</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1350</v>
       </c>
       <c r="C9" s="1">
-        <v>2390</v>
+        <v>4630</v>
       </c>
       <c r="D9" s="1">
-        <v>4770</v>
+        <v>9250</v>
       </c>
       <c r="E9" s="4">
         <f>(Table1[[#This Row],[requests per month]]-MIN(Table1[requests per month]))/(MAX(Table1[requests per month])-MIN(Table1[requests per month]))</f>
-        <v>3.0549236269093272E-3</v>
+        <v>3.2174195645108872E-2</v>
       </c>
       <c r="F9" s="5">
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
-        <v>1.1093023255813954</v>
-      </c>
-      <c r="G9" s="2">
-        <v>50.1</v>
-      </c>
-      <c r="H9" s="3">
+        <v>2.1511627906976742</v>
+      </c>
+      <c r="G9" s="6">
+        <v>42</v>
+      </c>
+      <c r="H9" s="6">
+        <v>60.8</v>
+      </c>
+      <c r="I9" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>1</v>
-      </c>
-      <c r="I9" s="2">
+        <v>0.50617283950617276</v>
+      </c>
+      <c r="J9" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.2945736434108526</v>
-      </c>
-      <c r="J9" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.50152746181345464</v>
+        <v>1.1558935361216729</v>
       </c>
       <c r="K9" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>0.26917351757564079</v>
+      </c>
+      <c r="L9" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>464848.91430934734</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+        <v>225244.9802630429</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B10" s="1">
-        <v>3200</v>
+        <v>4300</v>
       </c>
       <c r="C10" s="1">
-        <v>8000</v>
+        <v>10800</v>
       </c>
       <c r="D10" s="1">
-        <v>16000</v>
+        <v>21600</v>
       </c>
       <c r="E10" s="4">
         <f>(Table1[[#This Row],[requests per month]]-MIN(Table1[requests per month]))/(MAX(Table1[requests per month])-MIN(Table1[requests per month]))</f>
-        <v>7.6048098797530064E-2</v>
+        <v>0.11244718882027949</v>
       </c>
       <c r="F10" s="5">
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
-        <v>3.7209302325581395</v>
-      </c>
-      <c r="G10" s="2">
-        <v>43.4</v>
-      </c>
-      <c r="H10" s="3">
+        <v>5.0232558139534884</v>
+      </c>
+      <c r="G10" s="6">
+        <v>39</v>
+      </c>
+      <c r="H10" s="6">
+        <v>55.9</v>
+      </c>
+      <c r="I10" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0.41228070175438564</v>
-      </c>
-      <c r="I10" s="2">
+        <v>0.20370370370370358</v>
+      </c>
+      <c r="J10" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.1214470284237725</v>
-      </c>
-      <c r="J10" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.24416440027595784</v>
+        <v>1.0627376425855513</v>
       </c>
       <c r="K10" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>0.15807544626199155</v>
+      </c>
+      <c r="L10" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>276079.45502030326</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+        <v>207203.09320386467</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" s="1">
         <v>1150</v>
@@ -955,29 +1040,32 @@
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
         <v>1.3372093023255813</v>
       </c>
-      <c r="G11" s="2">
-        <v>47.1</v>
-      </c>
-      <c r="H11" s="3">
+      <c r="G11" s="6">
+        <v>44</v>
+      </c>
+      <c r="H11" s="6">
+        <v>61.8</v>
+      </c>
+      <c r="I11" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0.73684210526315785</v>
-      </c>
-      <c r="I11" s="2">
+        <v>0.56790123456790109</v>
+      </c>
+      <c r="J11" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.2170542635658914</v>
-      </c>
-      <c r="J11" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.37313343482202416</v>
+        <v>1.1749049429657794</v>
       </c>
       <c r="K11" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>0.28866299947439578</v>
+      </c>
+      <c r="L11" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>258106.47376137713</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+        <v>169334.99685100917</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="1">
         <v>3300</v>
@@ -996,29 +1084,32 @@
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
         <v>3.7906976744186047</v>
       </c>
-      <c r="G12" s="2">
-        <v>42.9</v>
-      </c>
-      <c r="H12" s="3">
+      <c r="G12" s="6">
+        <v>40</v>
+      </c>
+      <c r="H12" s="6">
+        <v>54.5</v>
+      </c>
+      <c r="I12" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0.36842105263157859</v>
-      </c>
-      <c r="I12" s="2">
+        <v>0.11728395061728389</v>
+      </c>
+      <c r="J12" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.1085271317829457</v>
-      </c>
-      <c r="J12" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.22320955134016368</v>
+        <v>1.0361216730038023</v>
       </c>
       <c r="K12" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>9.7641000333016342E-2</v>
+      </c>
+      <c r="L12" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>247167.47021932353</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+        <v>119822.50660230288</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" s="1">
         <v>3400</v>
@@ -1037,106 +1128,79 @@
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
         <v>3.9534883720930232</v>
       </c>
-      <c r="G13" s="2">
-        <v>41.9</v>
-      </c>
-      <c r="H13" s="3">
+      <c r="G13" s="6">
+        <v>38</v>
+      </c>
+      <c r="H13" s="6">
+        <v>52.6</v>
+      </c>
+      <c r="I13" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0.28070175438596456</v>
-      </c>
-      <c r="I13" s="2">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.0826873385012918</v>
-      </c>
-      <c r="J13" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.18162484534377851</v>
+        <v>1</v>
       </c>
       <c r="K13" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>4.1273968150796231E-2</v>
+      </c>
+      <c r="L13" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>199081.92578921453</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+        <v>87081.376398073073</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B14" s="1">
-        <v>1150</v>
+        <v>880</v>
       </c>
       <c r="C14" s="1">
-        <v>2880</v>
+        <v>2150</v>
       </c>
       <c r="D14" s="1">
-        <v>5750</v>
+        <v>4300</v>
       </c>
       <c r="E14" s="4">
         <f>(Table1[[#This Row],[requests per month]]-MIN(Table1[requests per month]))/(MAX(Table1[requests per month])-MIN(Table1[requests per month]))</f>
-        <v>9.4247643808904775E-3</v>
+        <v>0</v>
       </c>
       <c r="F14" s="5">
         <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
-        <v>1.3372093023255813</v>
-      </c>
-      <c r="G14" s="2">
-        <v>44.2</v>
-      </c>
-      <c r="H14" s="3">
+        <v>1</v>
+      </c>
+      <c r="G14" s="6">
+        <v>40</v>
+      </c>
+      <c r="H14" s="6">
+        <v>55.8</v>
+      </c>
+      <c r="I14" s="3">
         <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0.48245614035087725</v>
-      </c>
-      <c r="I14" s="2">
+        <v>0.19753086419753066</v>
+      </c>
+      <c r="J14" s="2">
         <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.1421188630490955</v>
-      </c>
-      <c r="J14" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.24594045236588385</v>
+        <v>1.0608365019011405</v>
       </c>
       <c r="K14" s="3">
+        <f>$B$17*Table1[[#This Row],[norm kota 5]]+$B$16*Table1[[#This Row],[norm kod]]</f>
+        <v>9.8765432098765329E-2</v>
+      </c>
+      <c r="L14" s="3">
         <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>121999.65094450633</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15">
-        <v>880</v>
-      </c>
-      <c r="C15" s="1">
-        <v>2150</v>
-      </c>
-      <c r="D15" s="1">
-        <v>4300</v>
-      </c>
-      <c r="E15" s="4">
-        <f>(Table1[[#This Row],[requests per month]]-MIN(Table1[requests per month]))/(MAX(Table1[requests per month])-MIN(Table1[requests per month]))</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="5">
-        <f>Table1[[#This Row],[requests per month]]/MIN(Table1[requests per month])</f>
-        <v>1</v>
-      </c>
-      <c r="G15" s="2">
-        <v>43.4</v>
-      </c>
-      <c r="H15" s="3">
-        <f>((Table1[[#This Row],[Coding]] - MIN(Table1[Coding])) / (MAX(Table1[Coding]) - MIN(Table1[Coding])))</f>
-        <v>0.41228070175438564</v>
-      </c>
-      <c r="I15" s="2">
-        <f>Table1[[#This Row],[Coding]]/ MIN(Table1[Coding])</f>
-        <v>1.1214470284237725</v>
-      </c>
-      <c r="J15" s="3">
-        <f>$B$18*Table1[[#This Row],[norm kota 5]]+$B$17*Table1[[#This Row],[norm kod]]</f>
-        <v>0.20614035087719282</v>
-      </c>
-      <c r="K15" s="3">
-        <f>Table1[[#This Row],[EK böl kota 6]]*EXP(Table1[[#This Row],[EK Böl Kod]]*10)</f>
-        <v>74196.353536706505</v>
+        <v>40471.974220948236</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>0.5</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -1144,65 +1208,238 @@
         <v>19</v>
       </c>
       <c r="B17">
+        <f>1-B16</f>
         <v>0.5</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18">
-        <f>1-B17</f>
-        <v>0.5</v>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <conditionalFormatting sqref="D1">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D14">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A3CE43A-694F-4F65-86E8-BFBA99593B09}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="6">
+        <v>40</v>
+      </c>
+      <c r="C2" s="6">
+        <v>56.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="6">
+        <v>44</v>
+      </c>
+      <c r="C3" s="6">
+        <v>59.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6">
+        <v>40</v>
+      </c>
+      <c r="C4" s="6">
+        <v>55.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="6">
+        <v>51</v>
+      </c>
+      <c r="C5" s="6">
+        <v>68.8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="6">
+        <v>44</v>
+      </c>
+      <c r="C6" s="6">
+        <v>61.8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="6">
+        <v>42</v>
+      </c>
+      <c r="C7" s="6">
+        <v>60.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="6">
+        <v>40</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="6">
+        <v>42</v>
+      </c>
+      <c r="C9" s="6">
+        <v>60.2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="6">
+        <v>38</v>
+      </c>
+      <c r="C10" s="6">
+        <v>52.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="6">
+        <v>44</v>
+      </c>
+      <c r="C11" s="6">
+        <v>58.6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="6">
+        <v>40</v>
+      </c>
+      <c r="C12" s="6">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="6">
+        <v>46</v>
+      </c>
+      <c r="C13" s="6">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="6">
+        <v>39</v>
+      </c>
+      <c r="C14" s="6">
+        <v>55.9</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>